<commit_message>
chore(export): regenerate 7-sheet workbook (corrected 5-level fills + sentiment-count consistency)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/exports/monthly_report.xlsx
+++ b/public/exports/monthly_report.xlsx
@@ -97,12 +97,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E7EBF0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
+        <fgColor rgb="00CFE8EF"/>
       </patternFill>
     </fill>
   </fills>
@@ -696,7 +696,7 @@
         <v>172</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>109</v>

</xml_diff>